<commit_message>
MARCATTA: corrige vínculo de custos dos componentes dos kits
</commit_message>
<xml_diff>
--- a/MARCATTA/MARCATTA_Fase_03_Catalogo_e_Precificacao_V1.0.xlsx
+++ b/MARCATTA/MARCATTA_Fase_03_Catalogo_e_Precificacao_V1.0.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="1" r:id="R466f344aacb24ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="2" r:id="Rec06d04d2ef04b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas" sheetId="3" r:id="Rb3f09b9304e24da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composição" sheetId="4" r:id="Rf26ddf52aa9f457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precificação" sheetId="5" r:id="R2431fe540ede48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="1" r:id="R8c5d7f9c5ecf48ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="2" r:id="R02261a9f852544d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas" sheetId="3" r:id="Rb12d8f16a047487e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composição" sheetId="4" r:id="Ra1cc9164b1234ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precificação" sheetId="5" r:id="R9fd2efc866b8403d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1769,7 +1769,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B7,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B7,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B7='Precificação'!A23,ISNUMBER('Precificação'!P23)),'Precificação'!P23,"")</x:f>
       </x:c>
       <x:c r="E7" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C7),C7&gt;0,ISNUMBER(D7)),C7*D7,"")</x:f>
@@ -1790,7 +1790,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B8,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B8,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B8='Precificação'!A24,ISNUMBER('Precificação'!P24)),'Precificação'!P24,"")</x:f>
       </x:c>
       <x:c r="E8" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C8),C8&gt;0,ISNUMBER(D8)),C8*D8,"")</x:f>
@@ -1811,7 +1811,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B9,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B9,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B9='Precificação'!A20,ISNUMBER('Precificação'!P20)),'Precificação'!P20,"")</x:f>
       </x:c>
       <x:c r="E9" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C9),C9&gt;0,ISNUMBER(D9)),C9*D9,"")</x:f>
@@ -1832,7 +1832,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B10,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B10,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B10='Precificação'!A21,ISNUMBER('Precificação'!P21)),'Precificação'!P21,"")</x:f>
       </x:c>
       <x:c r="E10" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C10),C10&gt;0,ISNUMBER(D10)),C10*D10,"")</x:f>
@@ -1853,7 +1853,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B11,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B11,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B11='Precificação'!A18,ISNUMBER('Precificação'!P18)),'Precificação'!P18,"")</x:f>
       </x:c>
       <x:c r="E11" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C11),C11&gt;0,ISNUMBER(D11)),C11*D11,"")</x:f>
@@ -1874,7 +1874,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B12,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B12,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B12='Precificação'!A23,ISNUMBER('Precificação'!P23)),'Precificação'!P23,"")</x:f>
       </x:c>
       <x:c r="E12" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C12),C12&gt;0,ISNUMBER(D12)),C12*D12,"")</x:f>
@@ -1895,7 +1895,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D13" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B13,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B13,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B13='Precificação'!A24,ISNUMBER('Precificação'!P24)),'Precificação'!P24,"")</x:f>
       </x:c>
       <x:c r="E13" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C13),C13&gt;0,ISNUMBER(D13)),C13*D13,"")</x:f>
@@ -1916,7 +1916,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B14,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B14,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B14='Precificação'!A17,ISNUMBER('Precificação'!P17)),'Precificação'!P17,"")</x:f>
       </x:c>
       <x:c r="E14" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C14),C14&gt;0,ISNUMBER(D14)),C14*D14,"")</x:f>
@@ -1937,7 +1937,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B15,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B15,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B15='Precificação'!A20,ISNUMBER('Precificação'!P20)),'Precificação'!P20,"")</x:f>
       </x:c>
       <x:c r="E15" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C15),C15&gt;0,ISNUMBER(D15)),C15*D15,"")</x:f>
@@ -1958,7 +1958,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B16,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B16,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B16='Precificação'!A22,ISNUMBER('Precificação'!P22)),'Precificação'!P22,"")</x:f>
       </x:c>
       <x:c r="E16" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C16),C16&gt;0,ISNUMBER(D16)),C16*D16,"")</x:f>
@@ -1979,7 +1979,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D17" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B17,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B17,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B17='Precificação'!A14,ISNUMBER('Precificação'!P14)),'Precificação'!P14,"")</x:f>
       </x:c>
       <x:c r="E17" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C17),C17&gt;0,ISNUMBER(D17)),C17*D17,"")</x:f>
@@ -2000,7 +2000,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D18" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B18,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B18,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B18='Precificação'!A12,ISNUMBER('Precificação'!P12)),'Precificação'!P12,"")</x:f>
       </x:c>
       <x:c r="E18" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C18),C18&gt;0,ISNUMBER(D18)),C18*D18,"")</x:f>
@@ -2021,7 +2021,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D19" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B19,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B19,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B19='Precificação'!A21,ISNUMBER('Precificação'!P21)),'Precificação'!P21,"")</x:f>
       </x:c>
       <x:c r="E19" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C19),C19&gt;0,ISNUMBER(D19)),C19*D19,"")</x:f>
@@ -2042,7 +2042,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D20" s="25" t="str">
-        <x:f>IFERROR(IF(ISNUMBER(VLOOKUP(B20,'Precificação'!$A$7:$P$24,16,FALSE)),VLOOKUP(B20,'Precificação'!$A$7:$P$24,16,FALSE),""),"")</x:f>
+        <x:f>IF(AND(B20='Precificação'!A24,ISNUMBER('Precificação'!P24)),'Precificação'!P24,"")</x:f>
       </x:c>
       <x:c r="E20" s="25" t="str">
         <x:f>IF(AND(ISNUMBER(C20),C20&gt;0,ISNUMBER(D20)),C20*D20,"")</x:f>

</xml_diff>